<commit_message>
แก้ test data Excel รอบ 2
</commit_message>
<xml_diff>
--- a/test_data/Test_Data_Downstream-for pilot.xlsx
+++ b/test_data/Test_Data_Downstream-for pilot.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="60" documentId="11_ACF12A4F8F533250C750CDEB4C3C9E6128049166" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C77C087A-42ED-4314-BA05-5794F1884A2D}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="114_{6BDDC0B5-1AE2-43CE-BA9D-EB249FA15F7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16542C7B-15B1-4E99-BCCE-B1C26AEC06AC}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="1296" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Data" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2026" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2005" uniqueCount="360">
   <si>
     <t>Template Test Case</t>
   </si>
@@ -1118,7 +1118,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="30" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1309,6 +1309,12 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="24">
@@ -1715,7 +1721,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1998,6 +2004,27 @@
     <xf numFmtId="0" fontId="28" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="29" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="28" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2010,25 +2037,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -2366,89 +2375,89 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:DB19"/>
-  <sheetFormatPr defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.08984375" customWidth="1"/>
-    <col min="2" max="2" width="13.453125" customWidth="1"/>
-    <col min="3" max="3" width="35.08984375" customWidth="1"/>
-    <col min="4" max="4" width="9.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.81640625" customWidth="1"/>
-    <col min="6" max="6" width="32.453125" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" customWidth="1"/>
+    <col min="1" max="1" width="4.140625" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" customWidth="1"/>
+    <col min="5" max="5" width="8.85546875" customWidth="1"/>
+    <col min="6" max="6" width="32.42578125" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="8.08984375" customWidth="1"/>
+    <col min="9" max="9" width="8.140625" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
     <col min="12" max="12" width="13" customWidth="1"/>
-    <col min="13" max="13" width="11.26953125" customWidth="1"/>
-    <col min="14" max="14" width="21.36328125" customWidth="1"/>
-    <col min="15" max="15" width="19.7265625" customWidth="1"/>
-    <col min="16" max="16" width="27.453125" customWidth="1"/>
-    <col min="17" max="17" width="25.08984375" customWidth="1"/>
+    <col min="13" max="13" width="11.28515625" customWidth="1"/>
+    <col min="14" max="14" width="21.42578125" customWidth="1"/>
+    <col min="15" max="15" width="19.7109375" customWidth="1"/>
+    <col min="16" max="16" width="27.42578125" customWidth="1"/>
+    <col min="17" max="17" width="25.140625" customWidth="1"/>
     <col min="18" max="18" width="11" customWidth="1"/>
-    <col min="19" max="19" width="21.7265625" customWidth="1"/>
-    <col min="20" max="20" width="12.54296875" customWidth="1"/>
-    <col min="21" max="21" width="31.08984375" customWidth="1"/>
-    <col min="22" max="22" width="16.453125" customWidth="1"/>
-    <col min="23" max="23" width="25.36328125" customWidth="1"/>
-    <col min="24" max="24" width="8.453125" customWidth="1"/>
-    <col min="25" max="25" width="15.36328125" customWidth="1"/>
-    <col min="26" max="26" width="14.81640625" customWidth="1"/>
-    <col min="27" max="27" width="15.36328125" customWidth="1"/>
-    <col min="28" max="28" width="16.81640625" customWidth="1"/>
-    <col min="29" max="29" width="19.453125" customWidth="1"/>
-    <col min="30" max="30" width="24.54296875" customWidth="1"/>
+    <col min="19" max="19" width="21.7109375" customWidth="1"/>
+    <col min="20" max="20" width="12.5703125" customWidth="1"/>
+    <col min="21" max="21" width="31.140625" customWidth="1"/>
+    <col min="22" max="22" width="16.42578125" customWidth="1"/>
+    <col min="23" max="23" width="25.42578125" customWidth="1"/>
+    <col min="24" max="24" width="8.42578125" customWidth="1"/>
+    <col min="25" max="25" width="15.42578125" customWidth="1"/>
+    <col min="26" max="26" width="14.85546875" customWidth="1"/>
+    <col min="27" max="27" width="15.42578125" customWidth="1"/>
+    <col min="28" max="28" width="16.85546875" customWidth="1"/>
+    <col min="29" max="29" width="19.42578125" customWidth="1"/>
+    <col min="30" max="30" width="24.5703125" customWidth="1"/>
     <col min="31" max="31" width="24" customWidth="1"/>
-    <col min="32" max="32" width="27.7265625" customWidth="1"/>
-    <col min="33" max="33" width="17.36328125" customWidth="1"/>
-    <col min="34" max="34" width="18.26953125" customWidth="1"/>
+    <col min="32" max="32" width="27.7109375" customWidth="1"/>
+    <col min="33" max="33" width="17.42578125" customWidth="1"/>
+    <col min="34" max="34" width="18.28515625" customWidth="1"/>
     <col min="35" max="35" width="24" customWidth="1"/>
-    <col min="36" max="36" width="16.26953125" customWidth="1"/>
+    <col min="36" max="36" width="16.28515625" customWidth="1"/>
     <col min="37" max="37" width="18" customWidth="1"/>
-    <col min="38" max="38" width="27.453125" customWidth="1"/>
-    <col min="39" max="39" width="21.36328125" customWidth="1"/>
-    <col min="40" max="40" width="15.26953125" customWidth="1"/>
+    <col min="38" max="38" width="27.42578125" customWidth="1"/>
+    <col min="39" max="39" width="21.42578125" customWidth="1"/>
+    <col min="40" max="40" width="15.28515625" customWidth="1"/>
     <col min="41" max="41" width="29" customWidth="1"/>
     <col min="42" max="42" width="22" customWidth="1"/>
-    <col min="43" max="43" width="8.08984375" customWidth="1"/>
+    <col min="43" max="43" width="8.140625" customWidth="1"/>
     <col min="44" max="44" width="11" customWidth="1"/>
-    <col min="45" max="45" width="14.36328125" customWidth="1"/>
-    <col min="46" max="46" width="23.36328125" customWidth="1"/>
-    <col min="47" max="47" width="23.08984375" customWidth="1"/>
-    <col min="48" max="48" width="17.453125" customWidth="1"/>
-    <col min="49" max="49" width="14.08984375" customWidth="1"/>
-    <col min="50" max="50" width="18.7265625" customWidth="1"/>
-    <col min="51" max="51" width="23.36328125" customWidth="1"/>
-    <col min="52" max="52" width="24.7265625" customWidth="1"/>
-    <col min="53" max="55" width="12.54296875" customWidth="1"/>
-    <col min="56" max="56" width="25.36328125" customWidth="1"/>
-    <col min="57" max="57" width="22.36328125" customWidth="1"/>
-    <col min="58" max="58" width="13.453125" customWidth="1"/>
-    <col min="59" max="59" width="15.08984375" customWidth="1"/>
-    <col min="60" max="60" width="13.36328125" customWidth="1"/>
-    <col min="61" max="61" width="14.36328125" customWidth="1"/>
-    <col min="62" max="62" width="15.36328125" customWidth="1"/>
-    <col min="63" max="63" width="17.81640625" customWidth="1"/>
-    <col min="64" max="64" width="12.54296875" customWidth="1"/>
-    <col min="65" max="65" width="27.36328125" customWidth="1"/>
-    <col min="66" max="66" width="24.36328125" customWidth="1"/>
-    <col min="67" max="73" width="12.54296875" customWidth="1"/>
-    <col min="74" max="74" width="27.36328125" customWidth="1"/>
-    <col min="75" max="75" width="24.36328125" customWidth="1"/>
-    <col min="76" max="87" width="12.54296875" customWidth="1"/>
-    <col min="88" max="88" width="15.7265625" customWidth="1"/>
-    <col min="89" max="95" width="12.54296875" customWidth="1"/>
-    <col min="96" max="96" width="15.7265625" customWidth="1"/>
-    <col min="97" max="97" width="17.7265625" customWidth="1"/>
-    <col min="98" max="98" width="19.54296875" customWidth="1"/>
+    <col min="45" max="45" width="14.42578125" customWidth="1"/>
+    <col min="46" max="46" width="23.42578125" customWidth="1"/>
+    <col min="47" max="47" width="23.140625" customWidth="1"/>
+    <col min="48" max="48" width="17.42578125" customWidth="1"/>
+    <col min="49" max="49" width="14.140625" customWidth="1"/>
+    <col min="50" max="50" width="18.7109375" customWidth="1"/>
+    <col min="51" max="51" width="23.42578125" customWidth="1"/>
+    <col min="52" max="52" width="24.7109375" customWidth="1"/>
+    <col min="53" max="55" width="12.5703125" customWidth="1"/>
+    <col min="56" max="56" width="25.42578125" customWidth="1"/>
+    <col min="57" max="57" width="22.42578125" customWidth="1"/>
+    <col min="58" max="58" width="13.42578125" customWidth="1"/>
+    <col min="59" max="59" width="15.140625" customWidth="1"/>
+    <col min="60" max="60" width="13.42578125" customWidth="1"/>
+    <col min="61" max="61" width="14.42578125" customWidth="1"/>
+    <col min="62" max="62" width="15.42578125" customWidth="1"/>
+    <col min="63" max="63" width="17.85546875" customWidth="1"/>
+    <col min="64" max="64" width="12.5703125" customWidth="1"/>
+    <col min="65" max="65" width="27.42578125" customWidth="1"/>
+    <col min="66" max="66" width="24.42578125" customWidth="1"/>
+    <col min="67" max="73" width="12.5703125" customWidth="1"/>
+    <col min="74" max="74" width="27.42578125" customWidth="1"/>
+    <col min="75" max="75" width="24.42578125" customWidth="1"/>
+    <col min="76" max="87" width="12.5703125" customWidth="1"/>
+    <col min="88" max="88" width="15.7109375" customWidth="1"/>
+    <col min="89" max="95" width="12.5703125" customWidth="1"/>
+    <col min="96" max="96" width="15.7109375" customWidth="1"/>
+    <col min="97" max="97" width="17.7109375" customWidth="1"/>
+    <col min="98" max="98" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:106" s="1" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:106" s="1" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:106" ht="6.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:106" s="3" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:106" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:106" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
@@ -2747,29 +2756,29 @@
         <v>98</v>
       </c>
     </row>
-    <row r="4" spans="1:106" s="7" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="N4" s="106" t="s">
+    <row r="4" spans="1:106" s="7" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N4" s="113" t="s">
         <v>2</v>
       </c>
-      <c r="O4" s="107"/>
-      <c r="P4" s="107"/>
-      <c r="Q4" s="107"/>
-      <c r="R4" s="107"/>
-      <c r="S4" s="107"/>
-      <c r="T4" s="107"/>
-      <c r="U4" s="107"/>
-      <c r="V4" s="107"/>
-      <c r="W4" s="107"/>
-      <c r="X4" s="107"/>
-      <c r="Y4" s="107"/>
-      <c r="Z4" s="107"/>
-      <c r="AA4" s="107"/>
-      <c r="AB4" s="107"/>
-      <c r="AC4" s="107"/>
-      <c r="AD4" s="107"/>
-      <c r="AE4" s="107"/>
-      <c r="AF4" s="107"/>
-      <c r="AG4" s="108"/>
+      <c r="O4" s="114"/>
+      <c r="P4" s="114"/>
+      <c r="Q4" s="114"/>
+      <c r="R4" s="114"/>
+      <c r="S4" s="114"/>
+      <c r="T4" s="114"/>
+      <c r="U4" s="114"/>
+      <c r="V4" s="114"/>
+      <c r="W4" s="114"/>
+      <c r="X4" s="114"/>
+      <c r="Y4" s="114"/>
+      <c r="Z4" s="114"/>
+      <c r="AA4" s="114"/>
+      <c r="AB4" s="114"/>
+      <c r="AC4" s="114"/>
+      <c r="AD4" s="114"/>
+      <c r="AE4" s="114"/>
+      <c r="AF4" s="114"/>
+      <c r="AG4" s="115"/>
       <c r="AH4" s="8" t="s">
         <v>3</v>
       </c>
@@ -2842,16 +2851,16 @@
       </c>
       <c r="CT4" s="13"/>
       <c r="CU4" s="13"/>
-      <c r="CW4" s="109" t="s">
+      <c r="CW4" s="116" t="s">
         <v>6</v>
       </c>
-      <c r="CX4" s="109"/>
-      <c r="CY4" s="109"/>
-      <c r="CZ4" s="109"/>
-      <c r="DA4" s="109"/>
-      <c r="DB4" s="109"/>
-    </row>
-    <row r="5" spans="1:106" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="CX4" s="116"/>
+      <c r="CY4" s="116"/>
+      <c r="CZ4" s="116"/>
+      <c r="DA4" s="116"/>
+      <c r="DB4" s="116"/>
+    </row>
+    <row r="5" spans="1:106" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="15"/>
       <c r="B5" s="16" t="s">
         <v>7</v>
@@ -3166,7 +3175,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:106" s="34" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="35"/>
       <c r="B6" s="36" t="s">
         <v>111</v>
@@ -3281,9 +3290,7 @@
       <c r="AO6" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="AP6" s="113" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP6" s="109"/>
       <c r="AQ6" s="38"/>
       <c r="AR6" s="38"/>
       <c r="AS6" s="38"/>
@@ -3291,7 +3298,7 @@
         <v>145</v>
       </c>
       <c r="AU6" s="38"/>
-      <c r="AV6" s="113"/>
+      <c r="AV6" s="109"/>
       <c r="AW6" s="38" t="s">
         <v>134</v>
       </c>
@@ -3382,7 +3389,7 @@
       <c r="DA6" s="46"/>
       <c r="DB6" s="46"/>
     </row>
-    <row r="7" spans="1:106" s="34" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="35"/>
       <c r="B7" s="36" t="s">
         <v>150</v>
@@ -3497,9 +3504,7 @@
       <c r="AO7" s="38" t="s">
         <v>173</v>
       </c>
-      <c r="AP7" s="113" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP7" s="109"/>
       <c r="AQ7" s="38"/>
       <c r="AR7" s="38"/>
       <c r="AS7" s="38"/>
@@ -3507,7 +3512,7 @@
         <v>145</v>
       </c>
       <c r="AU7" s="38"/>
-      <c r="AV7" s="113"/>
+      <c r="AV7" s="109"/>
       <c r="AW7" s="38" t="s">
         <v>174</v>
       </c>
@@ -3542,7 +3547,7 @@
       <c r="BJ7" s="38" t="s">
         <v>165</v>
       </c>
-      <c r="BK7" s="113"/>
+      <c r="BK7" s="109"/>
       <c r="BL7" s="38" t="s">
         <v>147</v>
       </c>
@@ -3555,7 +3560,7 @@
       <c r="BO7" s="50"/>
       <c r="BP7" s="50"/>
       <c r="BQ7" s="50"/>
-      <c r="BR7" s="113"/>
+      <c r="BR7" s="109"/>
       <c r="BS7" s="38"/>
       <c r="BT7" s="50"/>
       <c r="BU7" s="50"/>
@@ -3592,7 +3597,7 @@
       <c r="DA7" s="42"/>
       <c r="DB7" s="42"/>
     </row>
-    <row r="8" spans="1:106" s="34" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="B8" s="36" t="s">
         <v>177</v>
@@ -3704,9 +3709,7 @@
       <c r="AO8" s="38" t="s">
         <v>194</v>
       </c>
-      <c r="AP8" s="113" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP8" s="109"/>
       <c r="AQ8" s="38"/>
       <c r="AR8" s="38"/>
       <c r="AS8" s="38"/>
@@ -3714,7 +3717,7 @@
         <v>145</v>
       </c>
       <c r="AU8" s="38"/>
-      <c r="AV8" s="113"/>
+      <c r="AV8" s="109"/>
       <c r="AW8" s="38" t="s">
         <v>165</v>
       </c>
@@ -3749,7 +3752,7 @@
       <c r="BJ8" s="38" t="s">
         <v>187</v>
       </c>
-      <c r="BK8" s="113"/>
+      <c r="BK8" s="109"/>
       <c r="BL8" s="38" t="s">
         <v>147</v>
       </c>
@@ -3762,7 +3765,7 @@
       <c r="BO8" s="50"/>
       <c r="BP8" s="50"/>
       <c r="BQ8" s="50"/>
-      <c r="BR8" s="113"/>
+      <c r="BR8" s="109"/>
       <c r="BS8" s="38"/>
       <c r="BT8" s="50"/>
       <c r="BU8" s="50"/>
@@ -3799,7 +3802,7 @@
       <c r="DA8" s="42"/>
       <c r="DB8" s="42"/>
     </row>
-    <row r="9" spans="1:106" s="34" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="B9" s="36" t="s">
         <v>198</v>
@@ -3916,9 +3919,7 @@
       <c r="AO9" s="53" t="s">
         <v>214</v>
       </c>
-      <c r="AP9" s="113" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP9" s="109"/>
       <c r="AQ9" s="38"/>
       <c r="AR9" s="38"/>
       <c r="AS9" s="38"/>
@@ -3926,7 +3927,7 @@
         <v>145</v>
       </c>
       <c r="AU9" s="38"/>
-      <c r="AV9" s="113"/>
+      <c r="AV9" s="109"/>
       <c r="AW9" s="38" t="s">
         <v>174</v>
       </c>
@@ -4017,7 +4018,7 @@
       <c r="DA9" s="42"/>
       <c r="DB9" s="42"/>
     </row>
-    <row r="10" spans="1:106" s="34" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="35"/>
       <c r="B10" s="36" t="s">
         <v>217</v>
@@ -4042,36 +4043,32 @@
       <c r="J10" s="59"/>
       <c r="K10" s="59"/>
       <c r="L10" s="59"/>
-      <c r="M10" s="110"/>
-      <c r="N10" s="110"/>
-      <c r="O10" s="110"/>
+      <c r="M10" s="106"/>
+      <c r="N10" s="106"/>
+      <c r="O10" s="106"/>
       <c r="P10" s="59"/>
       <c r="Q10" s="59"/>
-      <c r="R10" s="110"/>
+      <c r="R10" s="106"/>
       <c r="S10" s="60" t="s">
         <v>220</v>
       </c>
       <c r="T10" s="59"/>
-      <c r="U10" s="110"/>
+      <c r="U10" s="106"/>
       <c r="V10" s="59"/>
       <c r="W10" s="59"/>
       <c r="X10" s="59"/>
-      <c r="Y10" s="110"/>
+      <c r="Y10" s="106"/>
       <c r="Z10" s="59"/>
       <c r="AA10" s="61" t="s">
         <v>139</v>
       </c>
       <c r="AB10" s="59"/>
-      <c r="AC10" s="112" t="s">
-        <v>144</v>
-      </c>
+      <c r="AC10" s="108"/>
       <c r="AD10" s="56">
         <v>0</v>
       </c>
       <c r="AE10" s="59"/>
-      <c r="AF10" s="110" t="s">
-        <v>144</v>
-      </c>
+      <c r="AF10" s="106"/>
       <c r="AG10" s="59"/>
       <c r="AH10" s="62">
         <v>0.32</v>
@@ -4081,33 +4078,29 @@
       </c>
       <c r="AJ10" s="59"/>
       <c r="AK10" s="59"/>
-      <c r="AL10" s="110" t="s">
-        <v>144</v>
-      </c>
+      <c r="AL10" s="106"/>
       <c r="AM10" s="59"/>
       <c r="AN10" s="59"/>
       <c r="AO10" s="63">
         <v>7775014694</v>
       </c>
-      <c r="AP10" s="110" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP10" s="106"/>
       <c r="AQ10" s="59"/>
       <c r="AR10" s="59"/>
       <c r="AS10" s="59"/>
       <c r="AT10" s="59"/>
       <c r="AU10" s="59"/>
-      <c r="AV10" s="110"/>
+      <c r="AV10" s="106"/>
       <c r="AW10" s="59" t="s">
         <v>139</v>
       </c>
       <c r="AX10" s="59"/>
-      <c r="AY10" s="110"/>
-      <c r="AZ10" s="110"/>
+      <c r="AY10" s="106"/>
+      <c r="AZ10" s="106"/>
       <c r="BA10" s="42"/>
-      <c r="BB10" s="116"/>
+      <c r="BB10" s="112"/>
       <c r="BC10" s="59"/>
-      <c r="BD10" s="116"/>
+      <c r="BD10" s="112"/>
       <c r="BE10" s="50"/>
       <c r="BF10" s="49"/>
       <c r="BG10" s="49"/>
@@ -4118,14 +4111,14 @@
       <c r="BJ10" s="65" t="s">
         <v>174</v>
       </c>
-      <c r="BK10" s="110"/>
+      <c r="BK10" s="106"/>
       <c r="BL10" s="59"/>
-      <c r="BM10" s="110"/>
+      <c r="BM10" s="106"/>
       <c r="BN10" s="50"/>
       <c r="BO10" s="50"/>
       <c r="BP10" s="50"/>
       <c r="BQ10" s="50"/>
-      <c r="BR10" s="110"/>
+      <c r="BR10" s="106"/>
       <c r="BS10" s="59"/>
       <c r="BT10" s="50"/>
       <c r="BU10" s="50"/>
@@ -4162,7 +4155,7 @@
       <c r="DA10" s="42"/>
       <c r="DB10" s="42"/>
     </row>
-    <row r="11" spans="1:106" s="34" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="66"/>
       <c r="B11" s="67" t="s">
         <v>222</v>
@@ -4285,9 +4278,7 @@
       <c r="AO11" s="68">
         <v>1233321</v>
       </c>
-      <c r="AP11" s="111" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP11" s="107"/>
       <c r="AQ11" s="68"/>
       <c r="AR11" s="68" t="s">
         <v>228</v>
@@ -4297,7 +4288,7 @@
         <v>145</v>
       </c>
       <c r="AU11" s="68"/>
-      <c r="AV11" s="111"/>
+      <c r="AV11" s="107"/>
       <c r="AW11" s="68" t="s">
         <v>174</v>
       </c>
@@ -4332,7 +4323,7 @@
       <c r="BJ11" s="68" t="s">
         <v>231</v>
       </c>
-      <c r="BK11" s="111"/>
+      <c r="BK11" s="107"/>
       <c r="BL11" s="68" t="s">
         <v>147</v>
       </c>
@@ -4345,7 +4336,7 @@
       <c r="BO11" s="50"/>
       <c r="BP11" s="50"/>
       <c r="BQ11" s="50"/>
-      <c r="BR11" s="111"/>
+      <c r="BR11" s="107"/>
       <c r="BS11" s="68"/>
       <c r="BT11" s="50"/>
       <c r="BU11" s="50"/>
@@ -4376,7 +4367,7 @@
       <c r="CT11" s="50"/>
       <c r="CU11" s="51"/>
     </row>
-    <row r="12" spans="1:106" s="34" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="71"/>
       <c r="B12" s="72" t="s">
         <v>234</v>
@@ -4499,9 +4490,7 @@
       <c r="AO12" s="68">
         <v>1234567</v>
       </c>
-      <c r="AP12" s="111" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP12" s="107"/>
       <c r="AQ12" s="68"/>
       <c r="AR12" s="68" t="s">
         <v>228</v>
@@ -4511,7 +4500,7 @@
         <v>145</v>
       </c>
       <c r="AU12" s="68"/>
-      <c r="AV12" s="111"/>
+      <c r="AV12" s="107"/>
       <c r="AW12" s="68" t="s">
         <v>174</v>
       </c>
@@ -4546,7 +4535,7 @@
       <c r="BJ12" s="74" t="s">
         <v>231</v>
       </c>
-      <c r="BK12" s="111"/>
+      <c r="BK12" s="107"/>
       <c r="BL12" s="68" t="s">
         <v>147</v>
       </c>
@@ -4559,7 +4548,7 @@
       <c r="BO12" s="50"/>
       <c r="BP12" s="50"/>
       <c r="BQ12" s="50"/>
-      <c r="BR12" s="111"/>
+      <c r="BR12" s="107"/>
       <c r="BS12" s="68" t="s">
         <v>228</v>
       </c>
@@ -4592,7 +4581,7 @@
       <c r="CT12" s="50"/>
       <c r="CU12" s="51"/>
     </row>
-    <row r="13" spans="1:106" s="34" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="71"/>
       <c r="B13" s="72" t="s">
         <v>243</v>
@@ -4715,9 +4704,7 @@
       <c r="AO13" s="75">
         <v>5643234</v>
       </c>
-      <c r="AP13" s="114" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP13" s="110"/>
       <c r="AQ13" s="75"/>
       <c r="AR13" s="75" t="s">
         <v>228</v>
@@ -4727,7 +4714,7 @@
         <v>145</v>
       </c>
       <c r="AU13" s="75"/>
-      <c r="AV13" s="114"/>
+      <c r="AV13" s="110"/>
       <c r="AW13" s="75" t="s">
         <v>134</v>
       </c>
@@ -4762,7 +4749,7 @@
       <c r="BJ13" s="75" t="s">
         <v>231</v>
       </c>
-      <c r="BK13" s="114"/>
+      <c r="BK13" s="110"/>
       <c r="BL13" s="75" t="s">
         <v>147</v>
       </c>
@@ -4775,7 +4762,7 @@
       <c r="BO13" s="50"/>
       <c r="BP13" s="50"/>
       <c r="BQ13" s="50"/>
-      <c r="BR13" s="111"/>
+      <c r="BR13" s="107"/>
       <c r="BS13" s="68" t="s">
         <v>228</v>
       </c>
@@ -4808,7 +4795,7 @@
       <c r="CT13" s="50"/>
       <c r="CU13" s="51"/>
     </row>
-    <row r="14" spans="1:106" s="34" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="71"/>
       <c r="B14" s="72" t="s">
         <v>250</v>
@@ -4931,9 +4918,7 @@
       <c r="AO14" s="68">
         <v>1234567</v>
       </c>
-      <c r="AP14" s="111" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP14" s="107"/>
       <c r="AQ14" s="68"/>
       <c r="AR14" s="68" t="s">
         <v>228</v>
@@ -4943,7 +4928,7 @@
         <v>145</v>
       </c>
       <c r="AU14" s="68"/>
-      <c r="AV14" s="111"/>
+      <c r="AV14" s="107"/>
       <c r="AW14" s="68" t="s">
         <v>174</v>
       </c>
@@ -4978,7 +4963,7 @@
       <c r="BJ14" s="68" t="s">
         <v>231</v>
       </c>
-      <c r="BK14" s="111"/>
+      <c r="BK14" s="107"/>
       <c r="BL14" s="68" t="s">
         <v>147</v>
       </c>
@@ -4991,7 +4976,7 @@
       <c r="BO14" s="50"/>
       <c r="BP14" s="50"/>
       <c r="BQ14" s="50"/>
-      <c r="BR14" s="111"/>
+      <c r="BR14" s="107"/>
       <c r="BS14" s="68"/>
       <c r="BT14" s="50"/>
       <c r="BU14" s="50"/>
@@ -5022,7 +5007,7 @@
       <c r="CT14" s="50"/>
       <c r="CU14" s="51"/>
     </row>
-    <row r="15" spans="1:106" s="34" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="71"/>
       <c r="B15" s="72" t="s">
         <v>256</v>
@@ -5145,9 +5130,7 @@
       <c r="AO15" s="75">
         <v>1234567</v>
       </c>
-      <c r="AP15" s="114" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP15" s="110"/>
       <c r="AQ15" s="75"/>
       <c r="AR15" s="75" t="s">
         <v>228</v>
@@ -5157,7 +5140,7 @@
         <v>145</v>
       </c>
       <c r="AU15" s="75"/>
-      <c r="AV15" s="114"/>
+      <c r="AV15" s="110"/>
       <c r="AW15" s="75" t="s">
         <v>139</v>
       </c>
@@ -5242,7 +5225,7 @@
       <c r="CT15" s="50"/>
       <c r="CU15" s="51"/>
     </row>
-    <row r="16" spans="1:106" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:106" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="77"/>
       <c r="B16" s="72" t="s">
         <v>265</v>
@@ -5356,9 +5339,7 @@
       <c r="AO16" s="78">
         <v>7776665</v>
       </c>
-      <c r="AP16" s="114" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP16" s="110"/>
       <c r="AQ16" s="81"/>
       <c r="AR16" s="81"/>
       <c r="AS16" s="81"/>
@@ -5401,14 +5382,14 @@
       <c r="BJ16" s="78" t="s">
         <v>187</v>
       </c>
-      <c r="BK16" s="111"/>
+      <c r="BK16" s="107"/>
       <c r="BL16" s="83"/>
-      <c r="BM16" s="111"/>
+      <c r="BM16" s="107"/>
       <c r="BN16" s="83"/>
       <c r="BO16" s="83"/>
       <c r="BP16" s="78"/>
       <c r="BQ16" s="78"/>
-      <c r="BR16" s="114"/>
+      <c r="BR16" s="110"/>
       <c r="BS16" s="78"/>
       <c r="BT16" s="82"/>
       <c r="BU16" s="78"/>
@@ -5439,7 +5420,7 @@
       <c r="CT16" s="81"/>
       <c r="CU16" s="81"/>
     </row>
-    <row r="17" spans="1:99" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:99" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="82"/>
       <c r="B17" s="36" t="s">
         <v>273</v>
@@ -5551,9 +5532,7 @@
       <c r="AO17" s="86">
         <v>6767679</v>
       </c>
-      <c r="AP17" s="115" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP17" s="111"/>
       <c r="AQ17" s="81"/>
       <c r="AR17" s="81"/>
       <c r="AS17" s="81"/>
@@ -5596,14 +5575,14 @@
       <c r="BJ17" s="86" t="s">
         <v>187</v>
       </c>
-      <c r="BK17" s="115"/>
+      <c r="BK17" s="111"/>
       <c r="BL17" s="86"/>
-      <c r="BM17" s="115"/>
+      <c r="BM17" s="111"/>
       <c r="BN17" s="86"/>
       <c r="BO17" s="86"/>
       <c r="BP17" s="86"/>
       <c r="BQ17" s="86"/>
-      <c r="BR17" s="115"/>
+      <c r="BR17" s="111"/>
       <c r="BS17" s="86"/>
       <c r="BT17" s="82"/>
       <c r="BU17" s="86"/>
@@ -5634,7 +5613,7 @@
       <c r="CT17" s="81"/>
       <c r="CU17" s="81"/>
     </row>
-    <row r="18" spans="1:99" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:99" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="89"/>
       <c r="B18" s="72" t="s">
         <v>281</v>
@@ -5746,9 +5725,7 @@
       <c r="AO18" s="90">
         <v>5656578</v>
       </c>
-      <c r="AP18" s="111" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP18" s="107"/>
       <c r="AQ18" s="92"/>
       <c r="AR18" s="92"/>
       <c r="AS18" s="92"/>
@@ -5791,14 +5768,14 @@
       <c r="BJ18" s="90" t="s">
         <v>187</v>
       </c>
-      <c r="BK18" s="111"/>
+      <c r="BK18" s="107"/>
       <c r="BL18" s="90"/>
-      <c r="BM18" s="111"/>
+      <c r="BM18" s="107"/>
       <c r="BN18" s="90"/>
       <c r="BO18" s="90"/>
       <c r="BP18" s="90"/>
       <c r="BQ18" s="90"/>
-      <c r="BR18" s="111"/>
+      <c r="BR18" s="107"/>
       <c r="BS18" s="90"/>
       <c r="BT18" s="93"/>
       <c r="BU18" s="90"/>
@@ -5829,7 +5806,7 @@
       <c r="CT18" s="92"/>
       <c r="CU18" s="92"/>
     </row>
-    <row r="19" spans="1:99" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:99" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="89"/>
       <c r="B19" s="96" t="s">
         <v>287</v>
@@ -5852,34 +5829,28 @@
       <c r="J19" s="90"/>
       <c r="K19" s="90"/>
       <c r="L19" s="90"/>
-      <c r="M19" s="111" t="s">
-        <v>144</v>
-      </c>
-      <c r="N19" s="111"/>
-      <c r="O19" s="111"/>
+      <c r="M19" s="117"/>
+      <c r="N19" s="107"/>
+      <c r="O19" s="107"/>
       <c r="P19" s="90"/>
       <c r="Q19" s="90"/>
-      <c r="R19" s="111"/>
-      <c r="S19" s="111"/>
+      <c r="R19" s="107"/>
+      <c r="S19" s="107"/>
       <c r="T19" s="90"/>
-      <c r="U19" s="111"/>
+      <c r="U19" s="107"/>
       <c r="V19" s="90"/>
       <c r="W19" s="90"/>
       <c r="X19" s="90"/>
-      <c r="Y19" s="111"/>
+      <c r="Y19" s="107"/>
       <c r="Z19" s="90"/>
-      <c r="AA19" s="111"/>
+      <c r="AA19" s="107"/>
       <c r="AB19" s="90"/>
       <c r="AC19" s="47">
         <v>769.16</v>
       </c>
-      <c r="AD19" s="111" t="s">
-        <v>144</v>
-      </c>
+      <c r="AD19" s="107"/>
       <c r="AE19" s="90"/>
-      <c r="AF19" s="111" t="s">
-        <v>144</v>
-      </c>
+      <c r="AF19" s="107"/>
       <c r="AG19" s="90"/>
       <c r="AH19" s="98">
         <v>65.09</v>
@@ -5889,31 +5860,27 @@
       </c>
       <c r="AJ19" s="90"/>
       <c r="AK19" s="90"/>
-      <c r="AL19" s="111" t="s">
-        <v>144</v>
-      </c>
+      <c r="AL19" s="107"/>
       <c r="AM19" s="90"/>
       <c r="AN19" s="90"/>
       <c r="AO19" s="90"/>
-      <c r="AP19" s="111" t="s">
-        <v>144</v>
-      </c>
+      <c r="AP19" s="107"/>
       <c r="AQ19" s="99"/>
       <c r="AR19" s="99"/>
       <c r="AS19" s="99"/>
       <c r="AT19" s="90"/>
       <c r="AU19" s="90"/>
-      <c r="AV19" s="111"/>
+      <c r="AV19" s="107"/>
       <c r="AW19" s="90"/>
       <c r="AX19" s="90"/>
-      <c r="AY19" s="111"/>
-      <c r="AZ19" s="111"/>
+      <c r="AY19" s="107"/>
+      <c r="AZ19" s="107"/>
       <c r="BA19" s="90"/>
       <c r="BB19" s="87" t="s">
         <v>146</v>
       </c>
       <c r="BC19" s="90"/>
-      <c r="BD19" s="111"/>
+      <c r="BD19" s="107"/>
       <c r="BE19" s="99"/>
       <c r="BF19" s="99"/>
       <c r="BG19" s="99"/>
@@ -5924,14 +5891,14 @@
       <c r="BJ19" s="98" t="s">
         <v>187</v>
       </c>
-      <c r="BK19" s="111"/>
+      <c r="BK19" s="107"/>
       <c r="BL19" s="90"/>
-      <c r="BM19" s="111"/>
+      <c r="BM19" s="107"/>
       <c r="BN19" s="90"/>
       <c r="BO19" s="90"/>
       <c r="BP19" s="90"/>
       <c r="BQ19" s="90"/>
-      <c r="BR19" s="111"/>
+      <c r="BR19" s="107"/>
       <c r="BS19" s="90"/>
       <c r="BT19" s="101"/>
       <c r="BU19" s="90"/>
@@ -5979,7 +5946,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E351"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
@@ -5988,7 +5955,7 @@
     <col min="5" max="5" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="102" t="s">
         <v>289</v>
       </c>
@@ -6005,7 +5972,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>6</v>
       </c>
@@ -6022,7 +5989,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>6</v>
       </c>
@@ -6039,7 +6006,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>6</v>
       </c>
@@ -6056,7 +6023,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>6</v>
       </c>
@@ -6073,7 +6040,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>6</v>
       </c>
@@ -6090,7 +6057,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -6107,7 +6074,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -6124,7 +6091,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>6</v>
       </c>
@@ -6141,7 +6108,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>6</v>
       </c>
@@ -6158,7 +6125,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>6</v>
       </c>
@@ -6175,7 +6142,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>6</v>
       </c>
@@ -6192,7 +6159,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>6</v>
       </c>
@@ -6209,7 +6176,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>6</v>
       </c>
@@ -6226,7 +6193,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>6</v>
       </c>
@@ -6243,7 +6210,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>6</v>
       </c>
@@ -6260,7 +6227,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>6</v>
       </c>
@@ -6277,7 +6244,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>6</v>
       </c>
@@ -6294,7 +6261,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>6</v>
       </c>
@@ -6311,7 +6278,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>6</v>
       </c>
@@ -6328,7 +6295,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>6</v>
       </c>
@@ -6345,7 +6312,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>6</v>
       </c>
@@ -6362,7 +6329,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>6</v>
       </c>
@@ -6379,7 +6346,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>6</v>
       </c>
@@ -6396,7 +6363,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>6</v>
       </c>
@@ -6413,7 +6380,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>6</v>
       </c>
@@ -6430,7 +6397,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>7</v>
       </c>
@@ -6447,7 +6414,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>7</v>
       </c>
@@ -6464,7 +6431,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>7</v>
       </c>
@@ -6481,7 +6448,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>7</v>
       </c>
@@ -6498,7 +6465,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>7</v>
       </c>
@@ -6515,7 +6482,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>7</v>
       </c>
@@ -6532,7 +6499,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>7</v>
       </c>
@@ -6549,7 +6516,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>7</v>
       </c>
@@ -6566,7 +6533,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>7</v>
       </c>
@@ -6583,7 +6550,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>7</v>
       </c>
@@ -6600,7 +6567,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>7</v>
       </c>
@@ -6617,7 +6584,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>7</v>
       </c>
@@ -6634,7 +6601,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>7</v>
       </c>
@@ -6651,7 +6618,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>7</v>
       </c>
@@ -6668,7 +6635,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>7</v>
       </c>
@@ -6685,7 +6652,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>7</v>
       </c>
@@ -6702,7 +6669,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>7</v>
       </c>
@@ -6719,7 +6686,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>7</v>
       </c>
@@ -6736,7 +6703,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>7</v>
       </c>
@@ -6753,7 +6720,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>7</v>
       </c>
@@ -6770,7 +6737,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>7</v>
       </c>
@@ -6787,7 +6754,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>7</v>
       </c>
@@ -6804,7 +6771,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>7</v>
       </c>
@@ -6821,7 +6788,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>7</v>
       </c>
@@ -6838,7 +6805,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>7</v>
       </c>
@@ -6855,7 +6822,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>8</v>
       </c>
@@ -6872,7 +6839,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>8</v>
       </c>
@@ -6889,7 +6856,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>8</v>
       </c>
@@ -6906,7 +6873,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>8</v>
       </c>
@@ -6923,7 +6890,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>8</v>
       </c>
@@ -6940,7 +6907,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>8</v>
       </c>
@@ -6957,7 +6924,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>8</v>
       </c>
@@ -6974,7 +6941,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>8</v>
       </c>
@@ -6991,7 +6958,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>8</v>
       </c>
@@ -7008,7 +6975,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>8</v>
       </c>
@@ -7025,7 +6992,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>8</v>
       </c>
@@ -7042,7 +7009,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>8</v>
       </c>
@@ -7059,7 +7026,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>8</v>
       </c>
@@ -7076,7 +7043,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>8</v>
       </c>
@@ -7093,7 +7060,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>8</v>
       </c>
@@ -7110,7 +7077,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>8</v>
       </c>
@@ -7127,7 +7094,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>8</v>
       </c>
@@ -7144,7 +7111,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>8</v>
       </c>
@@ -7161,7 +7128,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>8</v>
       </c>
@@ -7178,7 +7145,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>8</v>
       </c>
@@ -7195,7 +7162,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>8</v>
       </c>
@@ -7212,7 +7179,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>8</v>
       </c>
@@ -7229,7 +7196,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>8</v>
       </c>
@@ -7246,7 +7213,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>8</v>
       </c>
@@ -7263,7 +7230,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>8</v>
       </c>
@@ -7280,7 +7247,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>9</v>
       </c>
@@ -7297,7 +7264,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>9</v>
       </c>
@@ -7314,7 +7281,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>9</v>
       </c>
@@ -7331,7 +7298,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>9</v>
       </c>
@@ -7348,7 +7315,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>9</v>
       </c>
@@ -7365,7 +7332,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>9</v>
       </c>
@@ -7382,7 +7349,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>9</v>
       </c>
@@ -7399,7 +7366,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>9</v>
       </c>
@@ -7416,7 +7383,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>9</v>
       </c>
@@ -7433,7 +7400,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>9</v>
       </c>
@@ -7450,7 +7417,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>9</v>
       </c>
@@ -7467,7 +7434,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>9</v>
       </c>
@@ -7484,7 +7451,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>9</v>
       </c>
@@ -7501,7 +7468,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>9</v>
       </c>
@@ -7518,7 +7485,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>9</v>
       </c>
@@ -7535,7 +7502,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>9</v>
       </c>
@@ -7552,7 +7519,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>9</v>
       </c>
@@ -7569,7 +7536,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>9</v>
       </c>
@@ -7586,7 +7553,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>9</v>
       </c>
@@ -7603,7 +7570,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>9</v>
       </c>
@@ -7620,7 +7587,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>9</v>
       </c>
@@ -7637,7 +7604,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>9</v>
       </c>
@@ -7654,7 +7621,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>9</v>
       </c>
@@ -7671,7 +7638,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>9</v>
       </c>
@@ -7688,7 +7655,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>9</v>
       </c>
@@ -7705,7 +7672,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>10</v>
       </c>
@@ -7722,7 +7689,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>10</v>
       </c>
@@ -7739,7 +7706,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>10</v>
       </c>
@@ -7756,7 +7723,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>10</v>
       </c>
@@ -7773,7 +7740,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>10</v>
       </c>
@@ -7790,7 +7757,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>10</v>
       </c>
@@ -7807,7 +7774,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>10</v>
       </c>
@@ -7824,7 +7791,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>10</v>
       </c>
@@ -7841,7 +7808,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>10</v>
       </c>
@@ -7858,7 +7825,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>10</v>
       </c>
@@ -7875,7 +7842,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>10</v>
       </c>
@@ -7892,7 +7859,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>10</v>
       </c>
@@ -7909,7 +7876,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>10</v>
       </c>
@@ -7926,7 +7893,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>10</v>
       </c>
@@ -7943,7 +7910,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>10</v>
       </c>
@@ -7960,7 +7927,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>10</v>
       </c>
@@ -7977,7 +7944,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>10</v>
       </c>
@@ -7994,7 +7961,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>10</v>
       </c>
@@ -8011,7 +7978,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>10</v>
       </c>
@@ -8028,7 +7995,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>10</v>
       </c>
@@ -8045,7 +8012,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>10</v>
       </c>
@@ -8062,7 +8029,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>10</v>
       </c>
@@ -8079,7 +8046,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>10</v>
       </c>
@@ -8096,7 +8063,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>10</v>
       </c>
@@ -8113,7 +8080,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>10</v>
       </c>
@@ -8130,7 +8097,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>11</v>
       </c>
@@ -8147,7 +8114,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>11</v>
       </c>
@@ -8164,7 +8131,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>11</v>
       </c>
@@ -8181,7 +8148,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>11</v>
       </c>
@@ -8198,7 +8165,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>11</v>
       </c>
@@ -8215,7 +8182,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>11</v>
       </c>
@@ -8232,7 +8199,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>11</v>
       </c>
@@ -8249,7 +8216,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>11</v>
       </c>
@@ -8266,7 +8233,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>11</v>
       </c>
@@ -8283,7 +8250,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>11</v>
       </c>
@@ -8300,7 +8267,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>11</v>
       </c>
@@ -8317,7 +8284,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>11</v>
       </c>
@@ -8334,7 +8301,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>11</v>
       </c>
@@ -8351,7 +8318,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>11</v>
       </c>
@@ -8368,7 +8335,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>11</v>
       </c>
@@ -8385,7 +8352,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>11</v>
       </c>
@@ -8402,7 +8369,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>11</v>
       </c>
@@ -8419,7 +8386,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>11</v>
       </c>
@@ -8436,7 +8403,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>11</v>
       </c>
@@ -8453,7 +8420,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>11</v>
       </c>
@@ -8470,7 +8437,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>11</v>
       </c>
@@ -8487,7 +8454,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>11</v>
       </c>
@@ -8504,7 +8471,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>11</v>
       </c>
@@ -8521,7 +8488,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>11</v>
       </c>
@@ -8538,7 +8505,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>11</v>
       </c>
@@ -8555,7 +8522,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>12</v>
       </c>
@@ -8572,7 +8539,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>12</v>
       </c>
@@ -8589,7 +8556,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>12</v>
       </c>
@@ -8606,7 +8573,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>12</v>
       </c>
@@ -8623,7 +8590,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>12</v>
       </c>
@@ -8640,7 +8607,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>12</v>
       </c>
@@ -8657,7 +8624,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>12</v>
       </c>
@@ -8674,7 +8641,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>12</v>
       </c>
@@ -8691,7 +8658,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>12</v>
       </c>
@@ -8708,7 +8675,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>12</v>
       </c>
@@ -8725,7 +8692,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>12</v>
       </c>
@@ -8742,7 +8709,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>12</v>
       </c>
@@ -8759,7 +8726,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>12</v>
       </c>
@@ -8776,7 +8743,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>12</v>
       </c>
@@ -8793,7 +8760,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>12</v>
       </c>
@@ -8810,7 +8777,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>12</v>
       </c>
@@ -8827,7 +8794,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>12</v>
       </c>
@@ -8844,7 +8811,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>12</v>
       </c>
@@ -8861,7 +8828,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>12</v>
       </c>
@@ -8878,7 +8845,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>12</v>
       </c>
@@ -8895,7 +8862,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>12</v>
       </c>
@@ -8912,7 +8879,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>12</v>
       </c>
@@ -8929,7 +8896,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>12</v>
       </c>
@@ -8946,7 +8913,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>12</v>
       </c>
@@ -8963,7 +8930,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>12</v>
       </c>
@@ -8980,7 +8947,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>13</v>
       </c>
@@ -8997,7 +8964,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>13</v>
       </c>
@@ -9014,7 +8981,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>13</v>
       </c>
@@ -9031,7 +8998,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>13</v>
       </c>
@@ -9048,7 +9015,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>13</v>
       </c>
@@ -9065,7 +9032,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>13</v>
       </c>
@@ -9082,7 +9049,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>13</v>
       </c>
@@ -9099,7 +9066,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>13</v>
       </c>
@@ -9116,7 +9083,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>13</v>
       </c>
@@ -9133,7 +9100,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>13</v>
       </c>
@@ -9150,7 +9117,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>13</v>
       </c>
@@ -9167,7 +9134,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>13</v>
       </c>
@@ -9184,7 +9151,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>13</v>
       </c>
@@ -9201,7 +9168,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>13</v>
       </c>
@@ -9218,7 +9185,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>13</v>
       </c>
@@ -9235,7 +9202,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>13</v>
       </c>
@@ -9252,7 +9219,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>13</v>
       </c>
@@ -9269,7 +9236,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>13</v>
       </c>
@@ -9286,7 +9253,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>13</v>
       </c>
@@ -9303,7 +9270,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>13</v>
       </c>
@@ -9320,7 +9287,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>13</v>
       </c>
@@ -9337,7 +9304,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>13</v>
       </c>
@@ -9354,7 +9321,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>13</v>
       </c>
@@ -9371,7 +9338,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>13</v>
       </c>
@@ -9388,7 +9355,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>13</v>
       </c>
@@ -9405,7 +9372,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>14</v>
       </c>
@@ -9422,7 +9389,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>14</v>
       </c>
@@ -9439,7 +9406,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>14</v>
       </c>
@@ -9456,7 +9423,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>14</v>
       </c>
@@ -9473,7 +9440,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>14</v>
       </c>
@@ -9490,7 +9457,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>14</v>
       </c>
@@ -9507,7 +9474,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>14</v>
       </c>
@@ -9524,7 +9491,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>14</v>
       </c>
@@ -9541,7 +9508,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>14</v>
       </c>
@@ -9558,7 +9525,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>14</v>
       </c>
@@ -9575,7 +9542,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>14</v>
       </c>
@@ -9592,7 +9559,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>14</v>
       </c>
@@ -9609,7 +9576,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>14</v>
       </c>
@@ -9626,7 +9593,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>14</v>
       </c>
@@ -9643,7 +9610,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>14</v>
       </c>
@@ -9660,7 +9627,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>14</v>
       </c>
@@ -9677,7 +9644,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>14</v>
       </c>
@@ -9694,7 +9661,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>14</v>
       </c>
@@ -9711,7 +9678,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>14</v>
       </c>
@@ -9728,7 +9695,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>14</v>
       </c>
@@ -9745,7 +9712,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222">
         <v>14</v>
       </c>
@@ -9762,7 +9729,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223">
         <v>14</v>
       </c>
@@ -9779,7 +9746,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>14</v>
       </c>
@@ -9796,7 +9763,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>14</v>
       </c>
@@ -9813,7 +9780,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>14</v>
       </c>
@@ -9830,7 +9797,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>15</v>
       </c>
@@ -9847,7 +9814,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>15</v>
       </c>
@@ -9864,7 +9831,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>15</v>
       </c>
@@ -9881,7 +9848,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>15</v>
       </c>
@@ -9898,7 +9865,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>15</v>
       </c>
@@ -9915,7 +9882,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>15</v>
       </c>
@@ -9932,7 +9899,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233">
         <v>15</v>
       </c>
@@ -9949,7 +9916,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>15</v>
       </c>
@@ -9966,7 +9933,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>15</v>
       </c>
@@ -9983,7 +9950,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>15</v>
       </c>
@@ -10000,7 +9967,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>15</v>
       </c>
@@ -10017,7 +9984,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>15</v>
       </c>
@@ -10034,7 +10001,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>15</v>
       </c>
@@ -10051,7 +10018,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>15</v>
       </c>
@@ -10068,7 +10035,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>15</v>
       </c>
@@ -10085,7 +10052,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>15</v>
       </c>
@@ -10102,7 +10069,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243">
         <v>15</v>
       </c>
@@ -10119,7 +10086,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244">
         <v>15</v>
       </c>
@@ -10136,7 +10103,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>15</v>
       </c>
@@ -10153,7 +10120,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>15</v>
       </c>
@@ -10170,7 +10137,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>15</v>
       </c>
@@ -10187,7 +10154,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>15</v>
       </c>
@@ -10204,7 +10171,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249">
         <v>15</v>
       </c>
@@ -10221,7 +10188,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250">
         <v>15</v>
       </c>
@@ -10238,7 +10205,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251">
         <v>15</v>
       </c>
@@ -10255,7 +10222,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252">
         <v>16</v>
       </c>
@@ -10272,7 +10239,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253">
         <v>16</v>
       </c>
@@ -10289,7 +10256,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254">
         <v>16</v>
       </c>
@@ -10306,7 +10273,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255">
         <v>16</v>
       </c>
@@ -10323,7 +10290,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256">
         <v>16</v>
       </c>
@@ -10340,7 +10307,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257">
         <v>16</v>
       </c>
@@ -10357,7 +10324,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258">
         <v>16</v>
       </c>
@@ -10374,7 +10341,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259">
         <v>16</v>
       </c>
@@ -10391,7 +10358,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260">
         <v>16</v>
       </c>
@@ -10408,7 +10375,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261">
         <v>16</v>
       </c>
@@ -10425,7 +10392,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262">
         <v>16</v>
       </c>
@@ -10442,7 +10409,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263">
         <v>16</v>
       </c>
@@ -10459,7 +10426,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264">
         <v>16</v>
       </c>
@@ -10476,7 +10443,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265">
         <v>16</v>
       </c>
@@ -10493,7 +10460,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266">
         <v>16</v>
       </c>
@@ -10510,7 +10477,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267">
         <v>16</v>
       </c>
@@ -10527,7 +10494,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268">
         <v>16</v>
       </c>
@@ -10544,7 +10511,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269">
         <v>16</v>
       </c>
@@ -10561,7 +10528,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270">
         <v>16</v>
       </c>
@@ -10578,7 +10545,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271">
         <v>16</v>
       </c>
@@ -10595,7 +10562,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272">
         <v>16</v>
       </c>
@@ -10612,7 +10579,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273">
         <v>16</v>
       </c>
@@ -10629,7 +10596,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274">
         <v>16</v>
       </c>
@@ -10646,7 +10613,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275">
         <v>16</v>
       </c>
@@ -10663,7 +10630,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276">
         <v>16</v>
       </c>
@@ -10680,7 +10647,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277">
         <v>17</v>
       </c>
@@ -10697,7 +10664,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278">
         <v>17</v>
       </c>
@@ -10714,7 +10681,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279">
         <v>17</v>
       </c>
@@ -10731,7 +10698,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280">
         <v>17</v>
       </c>
@@ -10748,7 +10715,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281">
         <v>17</v>
       </c>
@@ -10765,7 +10732,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282">
         <v>17</v>
       </c>
@@ -10782,7 +10749,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A283">
         <v>17</v>
       </c>
@@ -10799,7 +10766,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284">
         <v>17</v>
       </c>
@@ -10816,7 +10783,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A285">
         <v>17</v>
       </c>
@@ -10833,7 +10800,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A286">
         <v>17</v>
       </c>
@@ -10850,7 +10817,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287">
         <v>17</v>
       </c>
@@ -10867,7 +10834,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A288">
         <v>17</v>
       </c>
@@ -10884,7 +10851,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289">
         <v>17</v>
       </c>
@@ -10901,7 +10868,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A290">
         <v>17</v>
       </c>
@@ -10918,7 +10885,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A291">
         <v>17</v>
       </c>
@@ -10935,7 +10902,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A292">
         <v>17</v>
       </c>
@@ -10952,7 +10919,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A293">
         <v>17</v>
       </c>
@@ -10969,7 +10936,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A294">
         <v>17</v>
       </c>
@@ -10986,7 +10953,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A295">
         <v>17</v>
       </c>
@@ -11003,7 +10970,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A296">
         <v>17</v>
       </c>
@@ -11020,7 +10987,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>17</v>
       </c>
@@ -11037,7 +11004,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>17</v>
       </c>
@@ -11054,7 +11021,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A299">
         <v>17</v>
       </c>
@@ -11071,7 +11038,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A300">
         <v>17</v>
       </c>
@@ -11088,7 +11055,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A301">
         <v>17</v>
       </c>
@@ -11105,7 +11072,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A302">
         <v>18</v>
       </c>
@@ -11122,7 +11089,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A303">
         <v>18</v>
       </c>
@@ -11139,7 +11106,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A304">
         <v>18</v>
       </c>
@@ -11156,7 +11123,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A305">
         <v>18</v>
       </c>
@@ -11173,7 +11140,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306">
         <v>18</v>
       </c>
@@ -11190,7 +11157,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A307">
         <v>18</v>
       </c>
@@ -11207,7 +11174,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A308">
         <v>18</v>
       </c>
@@ -11224,7 +11191,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A309">
         <v>18</v>
       </c>
@@ -11241,7 +11208,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A310">
         <v>18</v>
       </c>
@@ -11258,7 +11225,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A311">
         <v>18</v>
       </c>
@@ -11275,7 +11242,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A312">
         <v>18</v>
       </c>
@@ -11292,7 +11259,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A313">
         <v>18</v>
       </c>
@@ -11309,7 +11276,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A314">
         <v>18</v>
       </c>
@@ -11326,7 +11293,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A315">
         <v>18</v>
       </c>
@@ -11343,7 +11310,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A316">
         <v>18</v>
       </c>
@@ -11360,7 +11327,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A317">
         <v>18</v>
       </c>
@@ -11377,7 +11344,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A318">
         <v>18</v>
       </c>
@@ -11394,7 +11361,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A319">
         <v>18</v>
       </c>
@@ -11411,7 +11378,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A320">
         <v>18</v>
       </c>
@@ -11428,7 +11395,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A321">
         <v>18</v>
       </c>
@@ -11445,7 +11412,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A322">
         <v>18</v>
       </c>
@@ -11462,7 +11429,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A323">
         <v>18</v>
       </c>
@@ -11479,7 +11446,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A324">
         <v>18</v>
       </c>
@@ -11496,7 +11463,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A325">
         <v>18</v>
       </c>
@@ -11513,7 +11480,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A326">
         <v>18</v>
       </c>
@@ -11530,7 +11497,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A327">
         <v>19</v>
       </c>
@@ -11547,7 +11514,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A328">
         <v>19</v>
       </c>
@@ -11564,7 +11531,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A329">
         <v>19</v>
       </c>
@@ -11581,7 +11548,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A330">
         <v>19</v>
       </c>
@@ -11598,7 +11565,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A331">
         <v>19</v>
       </c>
@@ -11615,7 +11582,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A332">
         <v>19</v>
       </c>
@@ -11632,7 +11599,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A333">
         <v>19</v>
       </c>
@@ -11649,7 +11616,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A334">
         <v>19</v>
       </c>
@@ -11666,7 +11633,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A335">
         <v>19</v>
       </c>
@@ -11683,7 +11650,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A336">
         <v>19</v>
       </c>
@@ -11700,7 +11667,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A337">
         <v>19</v>
       </c>
@@ -11717,7 +11684,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A338">
         <v>19</v>
       </c>
@@ -11734,7 +11701,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A339">
         <v>19</v>
       </c>
@@ -11751,7 +11718,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A340">
         <v>19</v>
       </c>
@@ -11768,7 +11735,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A341">
         <v>19</v>
       </c>
@@ -11785,7 +11752,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A342">
         <v>19</v>
       </c>
@@ -11802,7 +11769,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A343">
         <v>19</v>
       </c>
@@ -11819,7 +11786,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A344">
         <v>19</v>
       </c>
@@ -11836,7 +11803,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A345">
         <v>19</v>
       </c>
@@ -11853,7 +11820,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A346">
         <v>19</v>
       </c>
@@ -11870,7 +11837,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A347">
         <v>19</v>
       </c>
@@ -11887,7 +11854,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A348">
         <v>19</v>
       </c>
@@ -11904,7 +11871,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A349">
         <v>19</v>
       </c>
@@ -11921,7 +11888,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A350">
         <v>19</v>
       </c>
@@ -11938,7 +11905,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A351">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
แก้ Logic highlight Header ของ PTX กับ LTX
</commit_message>
<xml_diff>
--- a/test_data/Test_Data_Downstream-for pilot.xlsx
+++ b/test_data/Test_Data_Downstream-for pilot.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="14" documentId="114_{6BDDC0B5-1AE2-43CE-BA9D-EB249FA15F7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2B22A1F-BF91-52E6-B2BC-B827D381FBB7}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="114_{6BDDC0B5-1AE2-43CE-BA9D-EB249FA15F7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE9510F7-D86D-4BCD-B4C1-0F5FAE124DEB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Data" sheetId="1" r:id="rId1"/>
@@ -1721,7 +1721,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2027,6 +2027,9 @@
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2379,89 +2382,89 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:DB19"/>
-  <sheetFormatPr defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.140625" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
-    <col min="3" max="3" width="35.140625" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" customWidth="1"/>
-    <col min="5" max="5" width="8.85546875" customWidth="1"/>
-    <col min="6" max="6" width="32.42578125" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" customWidth="1"/>
+    <col min="1" max="1" width="4.109375" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" customWidth="1"/>
+    <col min="3" max="3" width="35.109375" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" customWidth="1"/>
+    <col min="5" max="5" width="8.88671875" customWidth="1"/>
+    <col min="6" max="6" width="32.44140625" customWidth="1"/>
+    <col min="7" max="7" width="11.5546875" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="8.140625" customWidth="1"/>
+    <col min="9" max="9" width="8.109375" customWidth="1"/>
     <col min="10" max="10" width="11" customWidth="1"/>
     <col min="12" max="12" width="13" customWidth="1"/>
-    <col min="13" max="13" width="11.28515625" customWidth="1"/>
-    <col min="14" max="14" width="21.42578125" customWidth="1"/>
-    <col min="15" max="15" width="19.7109375" customWidth="1"/>
-    <col min="16" max="16" width="27.42578125" customWidth="1"/>
-    <col min="17" max="17" width="25.140625" customWidth="1"/>
+    <col min="13" max="13" width="11.33203125" customWidth="1"/>
+    <col min="14" max="14" width="21.44140625" customWidth="1"/>
+    <col min="15" max="15" width="19.6640625" customWidth="1"/>
+    <col min="16" max="16" width="27.44140625" customWidth="1"/>
+    <col min="17" max="17" width="25.109375" customWidth="1"/>
     <col min="18" max="18" width="11" customWidth="1"/>
-    <col min="19" max="19" width="21.7109375" customWidth="1"/>
-    <col min="20" max="20" width="12.5703125" customWidth="1"/>
-    <col min="21" max="21" width="31.140625" customWidth="1"/>
-    <col min="22" max="22" width="16.42578125" customWidth="1"/>
-    <col min="23" max="23" width="25.42578125" customWidth="1"/>
-    <col min="24" max="24" width="8.42578125" customWidth="1"/>
-    <col min="25" max="25" width="15.42578125" customWidth="1"/>
-    <col min="26" max="26" width="14.85546875" customWidth="1"/>
-    <col min="27" max="27" width="15.42578125" customWidth="1"/>
-    <col min="28" max="28" width="16.85546875" customWidth="1"/>
-    <col min="29" max="29" width="19.42578125" customWidth="1"/>
-    <col min="30" max="30" width="24.5703125" customWidth="1"/>
+    <col min="19" max="19" width="21.6640625" customWidth="1"/>
+    <col min="20" max="20" width="12.5546875" customWidth="1"/>
+    <col min="21" max="21" width="31.109375" customWidth="1"/>
+    <col min="22" max="22" width="16.44140625" customWidth="1"/>
+    <col min="23" max="23" width="25.44140625" customWidth="1"/>
+    <col min="24" max="24" width="8.44140625" customWidth="1"/>
+    <col min="25" max="25" width="15.44140625" customWidth="1"/>
+    <col min="26" max="26" width="14.88671875" customWidth="1"/>
+    <col min="27" max="27" width="15.44140625" customWidth="1"/>
+    <col min="28" max="28" width="16.88671875" customWidth="1"/>
+    <col min="29" max="29" width="19.44140625" customWidth="1"/>
+    <col min="30" max="30" width="24.5546875" customWidth="1"/>
     <col min="31" max="31" width="24" customWidth="1"/>
-    <col min="32" max="32" width="27.7109375" customWidth="1"/>
-    <col min="33" max="33" width="17.42578125" customWidth="1"/>
-    <col min="34" max="34" width="18.28515625" customWidth="1"/>
+    <col min="32" max="32" width="27.6640625" customWidth="1"/>
+    <col min="33" max="33" width="17.44140625" customWidth="1"/>
+    <col min="34" max="34" width="18.33203125" customWidth="1"/>
     <col min="35" max="35" width="24" customWidth="1"/>
-    <col min="36" max="36" width="16.28515625" customWidth="1"/>
+    <col min="36" max="36" width="16.33203125" customWidth="1"/>
     <col min="37" max="37" width="18" customWidth="1"/>
-    <col min="38" max="38" width="27.42578125" customWidth="1"/>
-    <col min="39" max="39" width="21.42578125" customWidth="1"/>
-    <col min="40" max="40" width="15.28515625" customWidth="1"/>
+    <col min="38" max="38" width="27.44140625" customWidth="1"/>
+    <col min="39" max="39" width="21.44140625" customWidth="1"/>
+    <col min="40" max="40" width="15.33203125" customWidth="1"/>
     <col min="41" max="41" width="29" customWidth="1"/>
     <col min="42" max="42" width="22" customWidth="1"/>
-    <col min="43" max="43" width="8.140625" customWidth="1"/>
+    <col min="43" max="43" width="8.109375" customWidth="1"/>
     <col min="44" max="44" width="11" customWidth="1"/>
-    <col min="45" max="45" width="14.42578125" customWidth="1"/>
-    <col min="46" max="46" width="23.42578125" customWidth="1"/>
-    <col min="47" max="47" width="23.140625" customWidth="1"/>
-    <col min="48" max="48" width="17.42578125" customWidth="1"/>
-    <col min="49" max="49" width="14.140625" customWidth="1"/>
-    <col min="50" max="50" width="18.7109375" customWidth="1"/>
-    <col min="51" max="51" width="23.42578125" customWidth="1"/>
-    <col min="52" max="52" width="24.7109375" customWidth="1"/>
-    <col min="53" max="55" width="12.5703125" customWidth="1"/>
-    <col min="56" max="56" width="25.42578125" customWidth="1"/>
-    <col min="57" max="57" width="22.42578125" customWidth="1"/>
-    <col min="58" max="58" width="13.42578125" customWidth="1"/>
-    <col min="59" max="59" width="15.140625" customWidth="1"/>
-    <col min="60" max="60" width="13.42578125" customWidth="1"/>
-    <col min="61" max="61" width="14.42578125" customWidth="1"/>
-    <col min="62" max="62" width="15.42578125" customWidth="1"/>
-    <col min="63" max="63" width="17.85546875" customWidth="1"/>
-    <col min="64" max="64" width="12.5703125" customWidth="1"/>
-    <col min="65" max="65" width="27.42578125" customWidth="1"/>
-    <col min="66" max="66" width="24.42578125" customWidth="1"/>
-    <col min="67" max="73" width="12.5703125" customWidth="1"/>
-    <col min="74" max="74" width="27.42578125" customWidth="1"/>
-    <col min="75" max="75" width="24.42578125" customWidth="1"/>
-    <col min="76" max="87" width="12.5703125" customWidth="1"/>
-    <col min="88" max="88" width="15.7109375" customWidth="1"/>
-    <col min="89" max="95" width="12.5703125" customWidth="1"/>
-    <col min="96" max="96" width="15.7109375" customWidth="1"/>
-    <col min="97" max="97" width="17.7109375" customWidth="1"/>
-    <col min="98" max="98" width="19.5703125" customWidth="1"/>
+    <col min="45" max="45" width="14.44140625" customWidth="1"/>
+    <col min="46" max="46" width="23.44140625" customWidth="1"/>
+    <col min="47" max="47" width="23.109375" customWidth="1"/>
+    <col min="48" max="48" width="17.44140625" customWidth="1"/>
+    <col min="49" max="49" width="14.109375" customWidth="1"/>
+    <col min="50" max="50" width="18.6640625" customWidth="1"/>
+    <col min="51" max="51" width="23.44140625" customWidth="1"/>
+    <col min="52" max="52" width="24.6640625" customWidth="1"/>
+    <col min="53" max="55" width="12.5546875" customWidth="1"/>
+    <col min="56" max="56" width="25.44140625" customWidth="1"/>
+    <col min="57" max="57" width="22.44140625" customWidth="1"/>
+    <col min="58" max="58" width="13.44140625" customWidth="1"/>
+    <col min="59" max="59" width="15.109375" customWidth="1"/>
+    <col min="60" max="60" width="13.44140625" customWidth="1"/>
+    <col min="61" max="61" width="14.44140625" customWidth="1"/>
+    <col min="62" max="62" width="15.44140625" customWidth="1"/>
+    <col min="63" max="63" width="17.88671875" customWidth="1"/>
+    <col min="64" max="64" width="12.5546875" customWidth="1"/>
+    <col min="65" max="65" width="27.44140625" customWidth="1"/>
+    <col min="66" max="66" width="24.44140625" customWidth="1"/>
+    <col min="67" max="73" width="12.5546875" customWidth="1"/>
+    <col min="74" max="74" width="27.44140625" customWidth="1"/>
+    <col min="75" max="75" width="24.44140625" customWidth="1"/>
+    <col min="76" max="87" width="12.5546875" customWidth="1"/>
+    <col min="88" max="88" width="15.6640625" customWidth="1"/>
+    <col min="89" max="95" width="12.5546875" customWidth="1"/>
+    <col min="96" max="96" width="15.6640625" customWidth="1"/>
+    <col min="97" max="97" width="17.6640625" customWidth="1"/>
+    <col min="98" max="98" width="19.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:106" s="1" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:106" s="1" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:106" ht="6.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:106" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:106" ht="6.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:106" s="3" customFormat="1" ht="16.8" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
@@ -2760,29 +2763,29 @@
         <v>98</v>
       </c>
     </row>
-    <row r="4" spans="1:106" s="7" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="N4" s="114" t="s">
+    <row r="4" spans="1:106" s="7" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="N4" s="115" t="s">
         <v>2</v>
       </c>
-      <c r="O4" s="115"/>
-      <c r="P4" s="115"/>
-      <c r="Q4" s="115"/>
-      <c r="R4" s="115"/>
-      <c r="S4" s="115"/>
-      <c r="T4" s="115"/>
-      <c r="U4" s="115"/>
-      <c r="V4" s="115"/>
-      <c r="W4" s="115"/>
-      <c r="X4" s="115"/>
-      <c r="Y4" s="115"/>
-      <c r="Z4" s="115"/>
-      <c r="AA4" s="115"/>
-      <c r="AB4" s="115"/>
-      <c r="AC4" s="115"/>
-      <c r="AD4" s="115"/>
-      <c r="AE4" s="115"/>
-      <c r="AF4" s="115"/>
-      <c r="AG4" s="116"/>
+      <c r="O4" s="116"/>
+      <c r="P4" s="116"/>
+      <c r="Q4" s="116"/>
+      <c r="R4" s="116"/>
+      <c r="S4" s="116"/>
+      <c r="T4" s="116"/>
+      <c r="U4" s="116"/>
+      <c r="V4" s="116"/>
+      <c r="W4" s="116"/>
+      <c r="X4" s="116"/>
+      <c r="Y4" s="116"/>
+      <c r="Z4" s="116"/>
+      <c r="AA4" s="116"/>
+      <c r="AB4" s="116"/>
+      <c r="AC4" s="116"/>
+      <c r="AD4" s="116"/>
+      <c r="AE4" s="116"/>
+      <c r="AF4" s="116"/>
+      <c r="AG4" s="117"/>
       <c r="AH4" s="8" t="s">
         <v>3</v>
       </c>
@@ -2855,16 +2858,16 @@
       </c>
       <c r="CT4" s="13"/>
       <c r="CU4" s="13"/>
-      <c r="CW4" s="117" t="s">
+      <c r="CW4" s="118" t="s">
         <v>6</v>
       </c>
-      <c r="CX4" s="117"/>
-      <c r="CY4" s="117"/>
-      <c r="CZ4" s="117"/>
-      <c r="DA4" s="117"/>
-      <c r="DB4" s="117"/>
-    </row>
-    <row r="5" spans="1:106" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="CX4" s="118"/>
+      <c r="CY4" s="118"/>
+      <c r="CZ4" s="118"/>
+      <c r="DA4" s="118"/>
+      <c r="DB4" s="118"/>
+    </row>
+    <row r="5" spans="1:106" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="15"/>
       <c r="B5" s="16" t="s">
         <v>7</v>
@@ -3179,7 +3182,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:106" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="35"/>
       <c r="B6" s="36" t="s">
         <v>111</v>
@@ -3393,7 +3396,7 @@
       <c r="DA6" s="46"/>
       <c r="DB6" s="46"/>
     </row>
-    <row r="7" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:106" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="35"/>
       <c r="B7" s="36" t="s">
         <v>150</v>
@@ -3601,7 +3604,7 @@
       <c r="DA7" s="42"/>
       <c r="DB7" s="42"/>
     </row>
-    <row r="8" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:106" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="35"/>
       <c r="B8" s="36" t="s">
         <v>177</v>
@@ -3775,7 +3778,7 @@
       <c r="BU8" s="50"/>
       <c r="BV8" s="50"/>
       <c r="BW8" s="50"/>
-      <c r="BX8" s="50"/>
+      <c r="BX8" s="114"/>
       <c r="BY8" s="50"/>
       <c r="BZ8" s="50"/>
       <c r="CA8" s="50"/>
@@ -3806,7 +3809,7 @@
       <c r="DA8" s="42"/>
       <c r="DB8" s="42"/>
     </row>
-    <row r="9" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:106" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="35"/>
       <c r="B9" s="36" t="s">
         <v>198</v>
@@ -3987,11 +3990,11 @@
       <c r="BS9" s="53" t="s">
         <v>174</v>
       </c>
-      <c r="BT9" s="50"/>
+      <c r="BT9" s="114"/>
       <c r="BU9" s="50"/>
       <c r="BV9" s="50"/>
       <c r="BW9" s="50"/>
-      <c r="BX9" s="50"/>
+      <c r="BX9" s="114"/>
       <c r="BY9" s="50"/>
       <c r="BZ9" s="50"/>
       <c r="CA9" s="50"/>
@@ -4022,7 +4025,7 @@
       <c r="DA9" s="42"/>
       <c r="DB9" s="42"/>
     </row>
-    <row r="10" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:106" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="35"/>
       <c r="B10" s="36" t="s">
         <v>217</v>
@@ -4159,7 +4162,7 @@
       <c r="DA10" s="42"/>
       <c r="DB10" s="42"/>
     </row>
-    <row r="11" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:106" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="66"/>
       <c r="B11" s="67" t="s">
         <v>222</v>
@@ -4371,7 +4374,7 @@
       <c r="CT11" s="50"/>
       <c r="CU11" s="51"/>
     </row>
-    <row r="12" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:106" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="71"/>
       <c r="B12" s="72" t="s">
         <v>234</v>
@@ -4558,7 +4561,7 @@
       </c>
       <c r="BT12" s="50"/>
       <c r="BU12" s="50"/>
-      <c r="BV12" s="50"/>
+      <c r="BV12" s="114"/>
       <c r="BW12" s="50"/>
       <c r="BX12" s="50"/>
       <c r="BY12" s="50"/>
@@ -4585,7 +4588,7 @@
       <c r="CT12" s="50"/>
       <c r="CU12" s="51"/>
     </row>
-    <row r="13" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:106" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="71"/>
       <c r="B13" s="72" t="s">
         <v>243</v>
@@ -4772,8 +4775,8 @@
       </c>
       <c r="BT13" s="50"/>
       <c r="BU13" s="50"/>
-      <c r="BV13" s="50"/>
-      <c r="BW13" s="50"/>
+      <c r="BV13" s="114"/>
+      <c r="BW13" s="114"/>
       <c r="BX13" s="50"/>
       <c r="BY13" s="50"/>
       <c r="BZ13" s="50"/>
@@ -4799,7 +4802,7 @@
       <c r="CT13" s="50"/>
       <c r="CU13" s="51"/>
     </row>
-    <row r="14" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:106" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="71"/>
       <c r="B14" s="72" t="s">
         <v>250</v>
@@ -5011,7 +5014,7 @@
       <c r="CT14" s="50"/>
       <c r="CU14" s="51"/>
     </row>
-    <row r="15" spans="1:106" s="34" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:106" s="34" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="71"/>
       <c r="B15" s="72" t="s">
         <v>256</v>
@@ -5229,7 +5232,7 @@
       <c r="CT15" s="50"/>
       <c r="CU15" s="51"/>
     </row>
-    <row r="16" spans="1:106" ht="15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:106" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A16" s="77"/>
       <c r="B16" s="72" t="s">
         <v>265</v>
@@ -5424,7 +5427,7 @@
       <c r="CT16" s="81"/>
       <c r="CU16" s="81"/>
     </row>
-    <row r="17" spans="1:99" ht="15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:99" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A17" s="82"/>
       <c r="B17" s="36" t="s">
         <v>273</v>
@@ -5617,7 +5620,7 @@
       <c r="CT17" s="81"/>
       <c r="CU17" s="81"/>
     </row>
-    <row r="18" spans="1:99" ht="15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:99" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18" s="89"/>
       <c r="B18" s="72" t="s">
         <v>281</v>
@@ -5810,7 +5813,7 @@
       <c r="CT18" s="92"/>
       <c r="CU18" s="92"/>
     </row>
-    <row r="19" spans="1:99" ht="15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:99" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19" s="89"/>
       <c r="B19" s="96" t="s">
         <v>287</v>
@@ -5950,7 +5953,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E351"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
@@ -5959,7 +5962,7 @@
     <col min="5" max="5" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="102" t="s">
         <v>289</v>
       </c>
@@ -5976,7 +5979,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>6</v>
       </c>
@@ -5993,7 +5996,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>6</v>
       </c>
@@ -6010,7 +6013,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>6</v>
       </c>
@@ -6027,7 +6030,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>6</v>
       </c>
@@ -6044,7 +6047,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
@@ -6061,7 +6064,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -6078,7 +6081,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -6095,7 +6098,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>6</v>
       </c>
@@ -6112,7 +6115,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>6</v>
       </c>
@@ -6129,7 +6132,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>6</v>
       </c>
@@ -6146,7 +6149,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>6</v>
       </c>
@@ -6163,7 +6166,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>6</v>
       </c>
@@ -6180,7 +6183,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>6</v>
       </c>
@@ -6197,7 +6200,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>6</v>
       </c>
@@ -6214,7 +6217,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>6</v>
       </c>
@@ -6231,7 +6234,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>6</v>
       </c>
@@ -6248,7 +6251,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>6</v>
       </c>
@@ -6265,7 +6268,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>6</v>
       </c>
@@ -6282,7 +6285,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>6</v>
       </c>
@@ -6299,7 +6302,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>6</v>
       </c>
@@ -6316,7 +6319,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>6</v>
       </c>
@@ -6333,7 +6336,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>6</v>
       </c>
@@ -6350,7 +6353,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>6</v>
       </c>
@@ -6367,7 +6370,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>6</v>
       </c>
@@ -6384,7 +6387,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>6</v>
       </c>
@@ -6401,7 +6404,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>7</v>
       </c>
@@ -6418,7 +6421,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>7</v>
       </c>
@@ -6435,7 +6438,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>7</v>
       </c>
@@ -6452,7 +6455,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>7</v>
       </c>
@@ -6469,7 +6472,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>7</v>
       </c>
@@ -6486,7 +6489,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>7</v>
       </c>
@@ -6503,7 +6506,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>7</v>
       </c>
@@ -6520,7 +6523,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>7</v>
       </c>
@@ -6537,7 +6540,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>7</v>
       </c>
@@ -6554,7 +6557,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>7</v>
       </c>
@@ -6571,7 +6574,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>7</v>
       </c>
@@ -6588,7 +6591,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>7</v>
       </c>
@@ -6605,7 +6608,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>7</v>
       </c>
@@ -6622,7 +6625,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>7</v>
       </c>
@@ -6639,7 +6642,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>7</v>
       </c>
@@ -6656,7 +6659,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>7</v>
       </c>
@@ -6673,7 +6676,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>7</v>
       </c>
@@ -6690,7 +6693,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>7</v>
       </c>
@@ -6707,7 +6710,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>7</v>
       </c>
@@ -6724,7 +6727,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>7</v>
       </c>
@@ -6741,7 +6744,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>7</v>
       </c>
@@ -6758,7 +6761,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>7</v>
       </c>
@@ -6775,7 +6778,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>7</v>
       </c>
@@ -6792,7 +6795,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>7</v>
       </c>
@@ -6809,7 +6812,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>7</v>
       </c>
@@ -6826,7 +6829,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>8</v>
       </c>
@@ -6843,7 +6846,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>8</v>
       </c>
@@ -6860,7 +6863,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>8</v>
       </c>
@@ -6877,7 +6880,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>8</v>
       </c>
@@ -6894,7 +6897,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>8</v>
       </c>
@@ -6911,7 +6914,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>8</v>
       </c>
@@ -6928,7 +6931,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>8</v>
       </c>
@@ -6945,7 +6948,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>8</v>
       </c>
@@ -6962,7 +6965,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>8</v>
       </c>
@@ -6979,7 +6982,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>8</v>
       </c>
@@ -6996,7 +6999,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>8</v>
       </c>
@@ -7013,7 +7016,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>8</v>
       </c>
@@ -7030,7 +7033,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>8</v>
       </c>
@@ -7047,7 +7050,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>8</v>
       </c>
@@ -7064,7 +7067,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>8</v>
       </c>
@@ -7081,7 +7084,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>8</v>
       </c>
@@ -7098,7 +7101,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>8</v>
       </c>
@@ -7115,7 +7118,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>8</v>
       </c>
@@ -7132,7 +7135,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>8</v>
       </c>
@@ -7149,7 +7152,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>8</v>
       </c>
@@ -7166,7 +7169,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>8</v>
       </c>
@@ -7183,7 +7186,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>8</v>
       </c>
@@ -7200,7 +7203,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>8</v>
       </c>
@@ -7217,7 +7220,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>8</v>
       </c>
@@ -7234,7 +7237,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>8</v>
       </c>
@@ -7251,7 +7254,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>9</v>
       </c>
@@ -7268,7 +7271,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>9</v>
       </c>
@@ -7285,7 +7288,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>9</v>
       </c>
@@ -7302,7 +7305,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>9</v>
       </c>
@@ -7319,7 +7322,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>9</v>
       </c>
@@ -7336,7 +7339,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>9</v>
       </c>
@@ -7353,7 +7356,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>9</v>
       </c>
@@ -7370,7 +7373,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>9</v>
       </c>
@@ -7387,7 +7390,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>9</v>
       </c>
@@ -7404,7 +7407,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>9</v>
       </c>
@@ -7421,7 +7424,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>9</v>
       </c>
@@ -7438,7 +7441,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>9</v>
       </c>
@@ -7455,7 +7458,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>9</v>
       </c>
@@ -7472,7 +7475,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>9</v>
       </c>
@@ -7489,7 +7492,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>9</v>
       </c>
@@ -7506,7 +7509,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>9</v>
       </c>
@@ -7523,7 +7526,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>9</v>
       </c>
@@ -7540,7 +7543,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>9</v>
       </c>
@@ -7557,7 +7560,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>9</v>
       </c>
@@ -7574,7 +7577,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>9</v>
       </c>
@@ -7591,7 +7594,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>9</v>
       </c>
@@ -7608,7 +7611,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>9</v>
       </c>
@@ -7625,7 +7628,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>9</v>
       </c>
@@ -7642,7 +7645,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>9</v>
       </c>
@@ -7659,7 +7662,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>9</v>
       </c>
@@ -7676,7 +7679,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>10</v>
       </c>
@@ -7693,7 +7696,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>10</v>
       </c>
@@ -7710,7 +7713,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>10</v>
       </c>
@@ -7727,7 +7730,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>10</v>
       </c>
@@ -7744,7 +7747,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>10</v>
       </c>
@@ -7761,7 +7764,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>10</v>
       </c>
@@ -7778,7 +7781,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>10</v>
       </c>
@@ -7795,7 +7798,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>10</v>
       </c>
@@ -7812,7 +7815,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>10</v>
       </c>
@@ -7829,7 +7832,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>10</v>
       </c>
@@ -7846,7 +7849,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>10</v>
       </c>
@@ -7863,7 +7866,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>10</v>
       </c>
@@ -7880,7 +7883,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>10</v>
       </c>
@@ -7897,7 +7900,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>10</v>
       </c>
@@ -7914,7 +7917,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>10</v>
       </c>
@@ -7931,7 +7934,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>10</v>
       </c>
@@ -7948,7 +7951,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>10</v>
       </c>
@@ -7965,7 +7968,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>10</v>
       </c>
@@ -7982,7 +7985,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>10</v>
       </c>
@@ -7999,7 +8002,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>10</v>
       </c>
@@ -8016,7 +8019,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>10</v>
       </c>
@@ -8033,7 +8036,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>10</v>
       </c>
@@ -8050,7 +8053,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>10</v>
       </c>
@@ -8067,7 +8070,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>10</v>
       </c>
@@ -8084,7 +8087,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>10</v>
       </c>
@@ -8101,7 +8104,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>11</v>
       </c>
@@ -8118,7 +8121,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>11</v>
       </c>
@@ -8135,7 +8138,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>11</v>
       </c>
@@ -8152,7 +8155,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>11</v>
       </c>
@@ -8169,7 +8172,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>11</v>
       </c>
@@ -8186,7 +8189,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>11</v>
       </c>
@@ -8203,7 +8206,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>11</v>
       </c>
@@ -8220,7 +8223,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>11</v>
       </c>
@@ -8237,7 +8240,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>11</v>
       </c>
@@ -8254,7 +8257,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>11</v>
       </c>
@@ -8271,7 +8274,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>11</v>
       </c>
@@ -8288,7 +8291,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>11</v>
       </c>
@@ -8305,7 +8308,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>11</v>
       </c>
@@ -8322,7 +8325,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>11</v>
       </c>
@@ -8339,7 +8342,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>11</v>
       </c>
@@ -8356,7 +8359,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>11</v>
       </c>
@@ -8373,7 +8376,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>11</v>
       </c>
@@ -8390,7 +8393,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>11</v>
       </c>
@@ -8407,7 +8410,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>11</v>
       </c>
@@ -8424,7 +8427,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>11</v>
       </c>
@@ -8441,7 +8444,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>11</v>
       </c>
@@ -8458,7 +8461,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>11</v>
       </c>
@@ -8475,7 +8478,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>11</v>
       </c>
@@ -8492,7 +8495,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>11</v>
       </c>
@@ -8509,7 +8512,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>11</v>
       </c>
@@ -8526,7 +8529,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>12</v>
       </c>
@@ -8543,7 +8546,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>12</v>
       </c>
@@ -8560,7 +8563,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>12</v>
       </c>
@@ -8577,7 +8580,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>12</v>
       </c>
@@ -8594,7 +8597,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>12</v>
       </c>
@@ -8611,7 +8614,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>12</v>
       </c>
@@ -8628,7 +8631,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>12</v>
       </c>
@@ -8645,7 +8648,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>12</v>
       </c>
@@ -8662,7 +8665,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>12</v>
       </c>
@@ -8679,7 +8682,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>12</v>
       </c>
@@ -8696,7 +8699,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>12</v>
       </c>
@@ -8713,7 +8716,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>12</v>
       </c>
@@ -8730,7 +8733,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>12</v>
       </c>
@@ -8747,7 +8750,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>12</v>
       </c>
@@ -8764,7 +8767,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>12</v>
       </c>
@@ -8781,7 +8784,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>12</v>
       </c>
@@ -8798,7 +8801,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>12</v>
       </c>
@@ -8815,7 +8818,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>12</v>
       </c>
@@ -8832,7 +8835,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>12</v>
       </c>
@@ -8849,7 +8852,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>12</v>
       </c>
@@ -8866,7 +8869,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>12</v>
       </c>
@@ -8883,7 +8886,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>12</v>
       </c>
@@ -8900,7 +8903,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>12</v>
       </c>
@@ -8917,7 +8920,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>12</v>
       </c>
@@ -8934,7 +8937,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>12</v>
       </c>
@@ -8951,7 +8954,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>13</v>
       </c>
@@ -8968,7 +8971,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>13</v>
       </c>
@@ -8985,7 +8988,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>13</v>
       </c>
@@ -9002,7 +9005,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>13</v>
       </c>
@@ -9019,7 +9022,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>13</v>
       </c>
@@ -9036,7 +9039,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>13</v>
       </c>
@@ -9053,7 +9056,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>13</v>
       </c>
@@ -9070,7 +9073,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>13</v>
       </c>
@@ -9087,7 +9090,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>13</v>
       </c>
@@ -9104,7 +9107,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>13</v>
       </c>
@@ -9121,7 +9124,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>13</v>
       </c>
@@ -9138,7 +9141,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>13</v>
       </c>
@@ -9155,7 +9158,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>13</v>
       </c>
@@ -9172,7 +9175,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>13</v>
       </c>
@@ -9189,7 +9192,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>13</v>
       </c>
@@ -9206,7 +9209,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>13</v>
       </c>
@@ -9223,7 +9226,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>13</v>
       </c>
@@ -9240,7 +9243,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>13</v>
       </c>
@@ -9257,7 +9260,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>13</v>
       </c>
@@ -9274,7 +9277,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>13</v>
       </c>
@@ -9291,7 +9294,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>13</v>
       </c>
@@ -9308,7 +9311,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>13</v>
       </c>
@@ -9325,7 +9328,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>13</v>
       </c>
@@ -9342,7 +9345,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>13</v>
       </c>
@@ -9359,7 +9362,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>13</v>
       </c>
@@ -9376,7 +9379,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>14</v>
       </c>
@@ -9393,7 +9396,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>14</v>
       </c>
@@ -9410,7 +9413,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>14</v>
       </c>
@@ -9427,7 +9430,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>14</v>
       </c>
@@ -9444,7 +9447,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>14</v>
       </c>
@@ -9461,7 +9464,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>14</v>
       </c>
@@ -9478,7 +9481,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>14</v>
       </c>
@@ -9495,7 +9498,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>14</v>
       </c>
@@ -9512,7 +9515,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>14</v>
       </c>
@@ -9529,7 +9532,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>14</v>
       </c>
@@ -9546,7 +9549,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>14</v>
       </c>
@@ -9563,7 +9566,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>14</v>
       </c>
@@ -9580,7 +9583,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>14</v>
       </c>
@@ -9597,7 +9600,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>14</v>
       </c>
@@ -9614,7 +9617,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>14</v>
       </c>
@@ -9631,7 +9634,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>14</v>
       </c>
@@ -9648,7 +9651,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>14</v>
       </c>
@@ -9665,7 +9668,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>14</v>
       </c>
@@ -9682,7 +9685,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>14</v>
       </c>
@@ -9699,7 +9702,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>14</v>
       </c>
@@ -9716,7 +9719,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>14</v>
       </c>
@@ -9733,7 +9736,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>14</v>
       </c>
@@ -9750,7 +9753,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>14</v>
       </c>
@@ -9767,7 +9770,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>14</v>
       </c>
@@ -9784,7 +9787,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>14</v>
       </c>
@@ -9801,7 +9804,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>15</v>
       </c>
@@ -9818,7 +9821,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>15</v>
       </c>
@@ -9835,7 +9838,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>15</v>
       </c>
@@ -9852,7 +9855,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>15</v>
       </c>
@@ -9869,7 +9872,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>15</v>
       </c>
@@ -9886,7 +9889,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>15</v>
       </c>
@@ -9903,7 +9906,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>15</v>
       </c>
@@ -9920,7 +9923,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>15</v>
       </c>
@@ -9937,7 +9940,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>15</v>
       </c>
@@ -9954,7 +9957,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>15</v>
       </c>
@@ -9971,7 +9974,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>15</v>
       </c>
@@ -9988,7 +9991,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>15</v>
       </c>
@@ -10005,7 +10008,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>15</v>
       </c>
@@ -10022,7 +10025,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>15</v>
       </c>
@@ -10039,7 +10042,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>15</v>
       </c>
@@ -10056,7 +10059,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>15</v>
       </c>
@@ -10073,7 +10076,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>15</v>
       </c>
@@ -10090,7 +10093,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>15</v>
       </c>
@@ -10107,7 +10110,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>15</v>
       </c>
@@ -10124,7 +10127,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>15</v>
       </c>
@@ -10141,7 +10144,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>15</v>
       </c>
@@ -10158,7 +10161,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>15</v>
       </c>
@@ -10175,7 +10178,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>15</v>
       </c>
@@ -10192,7 +10195,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>15</v>
       </c>
@@ -10209,7 +10212,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>15</v>
       </c>
@@ -10226,7 +10229,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>16</v>
       </c>
@@ -10243,7 +10246,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>16</v>
       </c>
@@ -10260,7 +10263,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>16</v>
       </c>
@@ -10277,7 +10280,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>16</v>
       </c>
@@ -10294,7 +10297,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>16</v>
       </c>
@@ -10311,7 +10314,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>16</v>
       </c>
@@ -10328,7 +10331,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>16</v>
       </c>
@@ -10345,7 +10348,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>16</v>
       </c>
@@ -10362,7 +10365,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>16</v>
       </c>
@@ -10379,7 +10382,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>16</v>
       </c>
@@ -10396,7 +10399,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>16</v>
       </c>
@@ -10413,7 +10416,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>16</v>
       </c>
@@ -10430,7 +10433,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>16</v>
       </c>
@@ -10447,7 +10450,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>16</v>
       </c>
@@ -10464,7 +10467,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>16</v>
       </c>
@@ -10481,7 +10484,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>16</v>
       </c>
@@ -10498,7 +10501,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>16</v>
       </c>
@@ -10515,7 +10518,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>16</v>
       </c>
@@ -10532,7 +10535,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>16</v>
       </c>
@@ -10549,7 +10552,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>16</v>
       </c>
@@ -10566,7 +10569,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>16</v>
       </c>
@@ -10583,7 +10586,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>16</v>
       </c>
@@ -10600,7 +10603,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>16</v>
       </c>
@@ -10617,7 +10620,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>16</v>
       </c>
@@ -10634,7 +10637,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>16</v>
       </c>
@@ -10651,7 +10654,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>17</v>
       </c>
@@ -10668,7 +10671,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>17</v>
       </c>
@@ -10685,7 +10688,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>17</v>
       </c>
@@ -10702,7 +10705,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>17</v>
       </c>
@@ -10719,7 +10722,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>17</v>
       </c>
@@ -10736,7 +10739,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>17</v>
       </c>
@@ -10753,7 +10756,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>17</v>
       </c>
@@ -10770,7 +10773,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>17</v>
       </c>
@@ -10787,7 +10790,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>17</v>
       </c>
@@ -10804,7 +10807,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>17</v>
       </c>
@@ -10821,7 +10824,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>17</v>
       </c>
@@ -10838,7 +10841,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>17</v>
       </c>
@@ -10855,7 +10858,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>17</v>
       </c>
@@ -10872,7 +10875,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>17</v>
       </c>
@@ -10889,7 +10892,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>17</v>
       </c>
@@ -10906,7 +10909,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>17</v>
       </c>
@@ -10923,7 +10926,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>17</v>
       </c>
@@ -10940,7 +10943,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>17</v>
       </c>
@@ -10957,7 +10960,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>17</v>
       </c>
@@ -10974,7 +10977,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>17</v>
       </c>
@@ -10991,7 +10994,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>17</v>
       </c>
@@ -11008,7 +11011,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>17</v>
       </c>
@@ -11025,7 +11028,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>17</v>
       </c>
@@ -11042,7 +11045,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>17</v>
       </c>
@@ -11059,7 +11062,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>17</v>
       </c>
@@ -11076,7 +11079,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>18</v>
       </c>
@@ -11093,7 +11096,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>18</v>
       </c>
@@ -11110,7 +11113,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>18</v>
       </c>
@@ -11127,7 +11130,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>18</v>
       </c>
@@ -11144,7 +11147,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>18</v>
       </c>
@@ -11161,7 +11164,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A307">
         <v>18</v>
       </c>
@@ -11178,7 +11181,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>18</v>
       </c>
@@ -11195,7 +11198,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A309">
         <v>18</v>
       </c>
@@ -11212,7 +11215,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A310">
         <v>18</v>
       </c>
@@ -11229,7 +11232,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A311">
         <v>18</v>
       </c>
@@ -11246,7 +11249,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A312">
         <v>18</v>
       </c>
@@ -11263,7 +11266,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>18</v>
       </c>
@@ -11280,7 +11283,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A314">
         <v>18</v>
       </c>
@@ -11297,7 +11300,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>18</v>
       </c>
@@ -11314,7 +11317,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A316">
         <v>18</v>
       </c>
@@ -11331,7 +11334,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A317">
         <v>18</v>
       </c>
@@ -11348,7 +11351,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>18</v>
       </c>
@@ -11365,7 +11368,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A319">
         <v>18</v>
       </c>
@@ -11382,7 +11385,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A320">
         <v>18</v>
       </c>
@@ -11399,7 +11402,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A321">
         <v>18</v>
       </c>
@@ -11416,7 +11419,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A322">
         <v>18</v>
       </c>
@@ -11433,7 +11436,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A323">
         <v>18</v>
       </c>
@@ -11450,7 +11453,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A324">
         <v>18</v>
       </c>
@@ -11467,7 +11470,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A325">
         <v>18</v>
       </c>
@@ -11484,7 +11487,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A326">
         <v>18</v>
       </c>
@@ -11501,7 +11504,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A327">
         <v>19</v>
       </c>
@@ -11518,7 +11521,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A328">
         <v>19</v>
       </c>
@@ -11535,7 +11538,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A329">
         <v>19</v>
       </c>
@@ -11552,7 +11555,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A330">
         <v>19</v>
       </c>
@@ -11569,7 +11572,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A331">
         <v>19</v>
       </c>
@@ -11586,7 +11589,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A332">
         <v>19</v>
       </c>
@@ -11603,7 +11606,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A333">
         <v>19</v>
       </c>
@@ -11620,7 +11623,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A334">
         <v>19</v>
       </c>
@@ -11637,7 +11640,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A335">
         <v>19</v>
       </c>
@@ -11654,7 +11657,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A336">
         <v>19</v>
       </c>
@@ -11671,7 +11674,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A337">
         <v>19</v>
       </c>
@@ -11688,7 +11691,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A338">
         <v>19</v>
       </c>
@@ -11705,7 +11708,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A339">
         <v>19</v>
       </c>
@@ -11722,7 +11725,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A340">
         <v>19</v>
       </c>
@@ -11739,7 +11742,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A341">
         <v>19</v>
       </c>
@@ -11756,7 +11759,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A342">
         <v>19</v>
       </c>
@@ -11773,7 +11776,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A343">
         <v>19</v>
       </c>
@@ -11790,7 +11793,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A344">
         <v>19</v>
       </c>
@@ -11807,7 +11810,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A345">
         <v>19</v>
       </c>
@@ -11824,7 +11827,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A346">
         <v>19</v>
       </c>
@@ -11841,7 +11844,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A347">
         <v>19</v>
       </c>
@@ -11858,7 +11861,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A348">
         <v>19</v>
       </c>
@@ -11875,7 +11878,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A349">
         <v>19</v>
       </c>
@@ -11892,7 +11895,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A350">
         <v>19</v>
       </c>
@@ -11909,7 +11912,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A351">
         <v>19</v>
       </c>

</xml_diff>